<commit_message>
fixes based on incorrect bom for cygnet mcu
</commit_message>
<xml_diff>
--- a/Cygnet/v1.2/Cygnet v1.2 BOM.xlsx
+++ b/Cygnet/v1.2/Cygnet v1.2 BOM.xlsx
@@ -558,13 +558,13 @@
     <t>STM32L433</t>
   </si>
   <si>
-    <t>Ultra-low-power with FPU ARM Cortex-M4 MCU 80 MHz with 128 Kbytes Flash, USB FS, LCD</t>
+    <t>Ultra-low-power with FPU ARM Cortex-M4 MCU 80 MHz with 256 Kbytes Flash, USB FS, LCD</t>
   </si>
   <si>
     <t>U1</t>
   </si>
   <si>
-    <t>STM32L433CB</t>
+    <t>STM32L433CCT6</t>
   </si>
   <si>
     <t>TPS63020DSJT</t>

</xml_diff>

<commit_message>
fixes based on incorrect bom for cygnet mcu (#46)
</commit_message>
<xml_diff>
--- a/Cygnet/v1.2/Cygnet v1.2 BOM.xlsx
+++ b/Cygnet/v1.2/Cygnet v1.2 BOM.xlsx
@@ -558,13 +558,13 @@
     <t>STM32L433</t>
   </si>
   <si>
-    <t>Ultra-low-power with FPU ARM Cortex-M4 MCU 80 MHz with 128 Kbytes Flash, USB FS, LCD</t>
+    <t>Ultra-low-power with FPU ARM Cortex-M4 MCU 80 MHz with 256 Kbytes Flash, USB FS, LCD</t>
   </si>
   <si>
     <t>U1</t>
   </si>
   <si>
-    <t>STM32L433CB</t>
+    <t>STM32L433CCT6</t>
   </si>
   <si>
     <t>TPS63020DSJT</t>

</xml_diff>